<commit_message>
no test multiple condition
</commit_message>
<xml_diff>
--- a/GameDisdockIP.xlsx
+++ b/GameDisdockIP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a34dfa97c331738/Documents/ilja/Unity/GMTK 2026 NEW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="443" documentId="8_{047D70A5-312B-42C2-AA54-1E0976B1220E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3BBDF79-7762-456D-8D3E-9DF5D5D767AB}"/>
+  <xr:revisionPtr revIDLastSave="447" documentId="8_{047D70A5-312B-42C2-AA54-1E0976B1220E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BE85B6C-4F72-4318-A74D-DB3D686B7333}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{11BF88F1-F4C2-45A5-8CCB-3492ED24BECA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="113">
   <si>
     <t>A</t>
   </si>
@@ -375,6 +375,9 @@
   </si>
   <si>
     <t>EE</t>
+  </si>
+  <si>
+    <t>if you palced card iwth n suits, grants vp for set</t>
   </si>
 </sst>
 </file>
@@ -815,7 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC38A9E3-0959-4F47-9569-6C1D59F951C2}">
-  <dimension ref="A1:AN49"/>
+  <dimension ref="A1:AN55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="12" max="12" width="11.28515625" customWidth="1"/>
@@ -2350,40 +2353,40 @@
       <c r="M31" s="7">
         <v>2</v>
       </c>
-      <c r="O31" s="9">
+      <c r="O31" s="6">
         <v>1</v>
       </c>
-      <c r="P31" s="9"/>
-      <c r="Q31" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="R31" s="11" t="s">
+      <c r="P31" s="6"/>
+      <c r="Q31" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="R31" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="S31" s="11"/>
-      <c r="T31" s="11"/>
-      <c r="U31" s="10">
+      <c r="S31" s="8"/>
+      <c r="T31" s="8"/>
+      <c r="U31" s="7">
         <v>25</v>
       </c>
-      <c r="V31" s="10">
-        <v>3</v>
-      </c>
-      <c r="X31" s="9">
+      <c r="V31" s="7">
+        <v>3</v>
+      </c>
+      <c r="X31" s="6">
         <v>1</v>
       </c>
-      <c r="Y31" s="9"/>
-      <c r="Z31" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="AA31" s="11" t="s">
+      <c r="Y31" s="6"/>
+      <c r="Z31" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA31" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="AB31" s="11"/>
-      <c r="AC31" s="11"/>
-      <c r="AD31" s="10">
+      <c r="AB31" s="8"/>
+      <c r="AC31" s="8"/>
+      <c r="AD31" s="7">
         <v>75</v>
       </c>
-      <c r="AE31" s="10">
+      <c r="AE31" s="7">
         <v>2</v>
       </c>
     </row>
@@ -2398,40 +2401,40 @@
       <c r="M32" s="7">
         <v>2</v>
       </c>
-      <c r="O32" s="9">
-        <v>2</v>
-      </c>
-      <c r="P32" s="9"/>
-      <c r="Q32" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="R32" s="11" t="s">
+      <c r="O32" s="6">
+        <v>2</v>
+      </c>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="R32" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="S32" s="11"/>
-      <c r="T32" s="11"/>
-      <c r="U32" s="10">
+      <c r="S32" s="8"/>
+      <c r="T32" s="8"/>
+      <c r="U32" s="7">
         <v>25</v>
       </c>
-      <c r="V32" s="10">
-        <v>3</v>
-      </c>
-      <c r="X32" s="9">
-        <v>2</v>
-      </c>
-      <c r="Y32" s="9"/>
-      <c r="Z32" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA32" s="11" t="s">
+      <c r="V32" s="7">
+        <v>3</v>
+      </c>
+      <c r="X32" s="6">
+        <v>2</v>
+      </c>
+      <c r="Y32" s="6"/>
+      <c r="Z32" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA32" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="AB32" s="11"/>
-      <c r="AC32" s="11"/>
-      <c r="AD32" s="10">
+      <c r="AB32" s="8"/>
+      <c r="AC32" s="8"/>
+      <c r="AD32" s="7">
         <v>75</v>
       </c>
-      <c r="AE32" s="10">
+      <c r="AE32" s="7">
         <v>2</v>
       </c>
     </row>
@@ -2454,40 +2457,40 @@
       <c r="M33" s="7">
         <v>2</v>
       </c>
-      <c r="O33" s="9">
-        <v>3</v>
-      </c>
-      <c r="P33" s="9"/>
-      <c r="Q33" s="10" t="s">
+      <c r="O33" s="6">
+        <v>3</v>
+      </c>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="R33" s="11" t="s">
+      <c r="R33" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="S33" s="11"/>
-      <c r="T33" s="11"/>
-      <c r="U33" s="10">
+      <c r="S33" s="8"/>
+      <c r="T33" s="8"/>
+      <c r="U33" s="7">
         <v>25</v>
       </c>
-      <c r="V33" s="10">
-        <v>3</v>
-      </c>
-      <c r="X33" s="9">
-        <v>3</v>
-      </c>
-      <c r="Y33" s="9"/>
-      <c r="Z33" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="AA33" s="11" t="s">
+      <c r="V33" s="7">
+        <v>3</v>
+      </c>
+      <c r="X33" s="6">
+        <v>3</v>
+      </c>
+      <c r="Y33" s="6"/>
+      <c r="Z33" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA33" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="AB33" s="11"/>
-      <c r="AC33" s="11"/>
-      <c r="AD33" s="9">
+      <c r="AB33" s="8"/>
+      <c r="AC33" s="8"/>
+      <c r="AD33" s="6">
         <v>125</v>
       </c>
-      <c r="AE33" s="10">
+      <c r="AE33" s="7">
         <v>2</v>
       </c>
     </row>
@@ -2502,40 +2505,40 @@
       <c r="M34" s="7">
         <v>2</v>
       </c>
-      <c r="O34" s="9">
+      <c r="O34" s="6">
         <v>4</v>
       </c>
-      <c r="P34" s="9"/>
-      <c r="Q34" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="R34" s="11" t="s">
+      <c r="P34" s="6"/>
+      <c r="Q34" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="R34" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="S34" s="11"/>
-      <c r="T34" s="11"/>
-      <c r="U34" s="10">
+      <c r="S34" s="8"/>
+      <c r="T34" s="8"/>
+      <c r="U34" s="7">
         <v>25</v>
       </c>
-      <c r="V34" s="10">
-        <v>3</v>
-      </c>
-      <c r="X34" s="9">
+      <c r="V34" s="7">
+        <v>3</v>
+      </c>
+      <c r="X34" s="6">
         <v>4</v>
       </c>
-      <c r="Y34" s="9"/>
-      <c r="Z34" s="10" t="s">
+      <c r="Y34" s="6"/>
+      <c r="Z34" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="AA34" s="11" t="s">
+      <c r="AA34" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="AB34" s="11"/>
-      <c r="AC34" s="11"/>
-      <c r="AD34" s="10">
+      <c r="AB34" s="8"/>
+      <c r="AC34" s="8"/>
+      <c r="AD34" s="7">
         <v>125</v>
       </c>
-      <c r="AE34" s="10">
+      <c r="AE34" s="7">
         <v>2</v>
       </c>
     </row>
@@ -2558,42 +2561,42 @@
       <c r="M35" s="7">
         <v>2</v>
       </c>
-      <c r="O35" s="9">
+      <c r="O35" s="6">
         <v>5</v>
       </c>
-      <c r="P35" s="9" t="s">
+      <c r="P35" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="Q35" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="R35" s="11" t="s">
+      <c r="Q35" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="R35" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="S35" s="11"/>
-      <c r="T35" s="11"/>
-      <c r="U35" s="10">
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
+      <c r="U35" s="7">
         <v>25</v>
       </c>
-      <c r="V35" s="10">
-        <v>3</v>
-      </c>
-      <c r="X35" s="9">
+      <c r="V35" s="7">
+        <v>3</v>
+      </c>
+      <c r="X35" s="6">
         <v>5</v>
       </c>
-      <c r="Y35" s="9"/>
-      <c r="Z35" s="10" t="s">
+      <c r="Y35" s="6"/>
+      <c r="Z35" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="AA35" s="11" t="s">
+      <c r="AA35" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="AB35" s="11"/>
-      <c r="AC35" s="11"/>
-      <c r="AD35" s="10">
+      <c r="AB35" s="8"/>
+      <c r="AC35" s="8"/>
+      <c r="AD35" s="7">
         <v>175</v>
       </c>
-      <c r="AE35" s="10">
+      <c r="AE35" s="7">
         <v>3</v>
       </c>
     </row>
@@ -2608,40 +2611,40 @@
       <c r="M36" s="7">
         <v>2</v>
       </c>
-      <c r="O36" s="9">
+      <c r="O36" s="6">
         <v>6</v>
       </c>
-      <c r="P36" s="9"/>
-      <c r="Q36" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="R36" s="11" t="s">
+      <c r="P36" s="6"/>
+      <c r="Q36" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="R36" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="S36" s="11"/>
-      <c r="T36" s="11"/>
-      <c r="U36" s="10">
+      <c r="S36" s="8"/>
+      <c r="T36" s="8"/>
+      <c r="U36" s="7">
         <v>25</v>
       </c>
-      <c r="V36" s="10">
+      <c r="V36" s="7">
         <v>4</v>
       </c>
-      <c r="X36" s="9">
+      <c r="X36" s="6">
         <v>6</v>
       </c>
-      <c r="Y36" s="9"/>
-      <c r="Z36" s="10" t="s">
+      <c r="Y36" s="6"/>
+      <c r="Z36" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="AA36" s="11" t="s">
+      <c r="AA36" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="AB36" s="11"/>
-      <c r="AC36" s="11"/>
-      <c r="AD36" s="10">
+      <c r="AB36" s="8"/>
+      <c r="AC36" s="8"/>
+      <c r="AD36" s="7">
         <v>670</v>
       </c>
-      <c r="AE36" s="10">
+      <c r="AE36" s="7">
         <v>3</v>
       </c>
     </row>
@@ -2664,40 +2667,40 @@
       <c r="M37" s="7">
         <v>2</v>
       </c>
-      <c r="O37" s="9">
+      <c r="O37" s="6">
         <v>7</v>
       </c>
-      <c r="P37" s="9"/>
-      <c r="Q37" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="R37" s="11" t="s">
+      <c r="P37" s="6"/>
+      <c r="Q37" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="R37" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="S37" s="11"/>
-      <c r="T37" s="11"/>
-      <c r="U37" s="10">
+      <c r="S37" s="8"/>
+      <c r="T37" s="8"/>
+      <c r="U37" s="7">
         <v>25</v>
       </c>
-      <c r="V37" s="10">
-        <v>3</v>
-      </c>
-      <c r="X37" s="9">
+      <c r="V37" s="7">
+        <v>3</v>
+      </c>
+      <c r="X37" s="6">
         <v>7</v>
       </c>
-      <c r="Y37" s="9"/>
-      <c r="Z37" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="AA37" s="11" t="s">
+      <c r="Y37" s="6"/>
+      <c r="Z37" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA37" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="AB37" s="11"/>
-      <c r="AC37" s="11"/>
-      <c r="AD37" s="10">
+      <c r="AB37" s="8"/>
+      <c r="AC37" s="8"/>
+      <c r="AD37" s="7">
         <v>75</v>
       </c>
-      <c r="AE37" s="10"/>
+      <c r="AE37" s="7"/>
     </row>
     <row r="38" spans="6:31" x14ac:dyDescent="0.25">
       <c r="F38" s="6"/>
@@ -2710,40 +2713,40 @@
       <c r="M38" s="7">
         <v>2</v>
       </c>
-      <c r="O38" s="9">
+      <c r="O38" s="6">
         <v>8</v>
       </c>
-      <c r="P38" s="9"/>
-      <c r="Q38" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="R38" s="11" t="s">
+      <c r="P38" s="6"/>
+      <c r="Q38" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="R38" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="S38" s="11"/>
-      <c r="T38" s="11"/>
-      <c r="U38" s="10">
+      <c r="S38" s="8"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="7">
         <v>50</v>
       </c>
-      <c r="V38" s="10">
-        <v>3</v>
-      </c>
-      <c r="X38" s="9">
+      <c r="V38" s="7">
+        <v>3</v>
+      </c>
+      <c r="X38" s="6">
         <v>8</v>
       </c>
-      <c r="Y38" s="9"/>
-      <c r="Z38" s="10" t="s">
+      <c r="Y38" s="6"/>
+      <c r="Z38" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="AA38" s="11" t="s">
+      <c r="AA38" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="AB38" s="11"/>
-      <c r="AC38" s="11"/>
-      <c r="AD38" s="10">
+      <c r="AB38" s="8"/>
+      <c r="AC38" s="8"/>
+      <c r="AD38" s="7">
         <v>75</v>
       </c>
-      <c r="AE38" s="10"/>
+      <c r="AE38" s="7"/>
     </row>
     <row r="39" spans="6:31" x14ac:dyDescent="0.25">
       <c r="F39" s="6">
@@ -2764,40 +2767,40 @@
       <c r="M39" s="7">
         <v>2</v>
       </c>
-      <c r="O39" s="9">
+      <c r="O39" s="6">
         <v>9</v>
       </c>
-      <c r="P39" s="9"/>
-      <c r="Q39" s="10" t="s">
+      <c r="P39" s="6"/>
+      <c r="Q39" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="R39" s="11" t="s">
+      <c r="R39" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="S39" s="11"/>
-      <c r="T39" s="11"/>
-      <c r="U39" s="10">
+      <c r="S39" s="8"/>
+      <c r="T39" s="8"/>
+      <c r="U39" s="7">
         <v>75</v>
       </c>
-      <c r="V39" s="10">
-        <v>3</v>
-      </c>
-      <c r="X39" s="9">
+      <c r="V39" s="7">
+        <v>3</v>
+      </c>
+      <c r="X39" s="6">
         <v>9</v>
       </c>
-      <c r="Y39" s="9"/>
-      <c r="Z39" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="AA39" s="11" t="s">
+      <c r="Y39" s="6"/>
+      <c r="Z39" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA39" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="AB39" s="11"/>
-      <c r="AC39" s="11"/>
-      <c r="AD39" s="10">
+      <c r="AB39" s="8"/>
+      <c r="AC39" s="8"/>
+      <c r="AD39" s="7">
         <v>125</v>
       </c>
-      <c r="AE39" s="10"/>
+      <c r="AE39" s="7"/>
     </row>
     <row r="40" spans="6:31" x14ac:dyDescent="0.25">
       <c r="F40" s="6"/>
@@ -2810,40 +2813,40 @@
       <c r="M40" s="7">
         <v>2</v>
       </c>
-      <c r="O40" s="9">
+      <c r="O40" s="6">
         <v>10</v>
       </c>
-      <c r="P40" s="9"/>
-      <c r="Q40" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="R40" s="11" t="s">
+      <c r="P40" s="6"/>
+      <c r="Q40" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="R40" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="S40" s="11"/>
-      <c r="T40" s="11"/>
-      <c r="U40" s="10">
+      <c r="S40" s="8"/>
+      <c r="T40" s="8"/>
+      <c r="U40" s="7">
         <v>25</v>
       </c>
-      <c r="V40" s="10">
+      <c r="V40" s="7">
         <v>4</v>
       </c>
-      <c r="X40" s="9">
+      <c r="X40" s="6">
         <v>10</v>
       </c>
-      <c r="Y40" s="9"/>
-      <c r="Z40" s="10" t="s">
+      <c r="Y40" s="6"/>
+      <c r="Z40" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="AA40" s="11" t="s">
+      <c r="AA40" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="AB40" s="11"/>
-      <c r="AC40" s="11"/>
-      <c r="AD40" s="10">
+      <c r="AB40" s="8"/>
+      <c r="AC40" s="8"/>
+      <c r="AD40" s="7">
         <v>125</v>
       </c>
-      <c r="AE40" s="10"/>
+      <c r="AE40" s="7"/>
     </row>
     <row r="41" spans="6:31" x14ac:dyDescent="0.25">
       <c r="F41" s="6">
@@ -2864,40 +2867,40 @@
       <c r="M41" s="7">
         <v>3</v>
       </c>
-      <c r="O41" s="9">
+      <c r="O41" s="6">
         <v>11</v>
       </c>
-      <c r="P41" s="9"/>
-      <c r="Q41" s="10" t="s">
+      <c r="P41" s="6"/>
+      <c r="Q41" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="R41" s="11" t="s">
+      <c r="R41" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="S41" s="11"/>
-      <c r="T41" s="11"/>
-      <c r="U41" s="10">
+      <c r="S41" s="8"/>
+      <c r="T41" s="8"/>
+      <c r="U41" s="7">
         <v>25</v>
       </c>
-      <c r="V41" s="10">
-        <v>3</v>
-      </c>
-      <c r="X41" s="9">
+      <c r="V41" s="7">
+        <v>3</v>
+      </c>
+      <c r="X41" s="6">
         <v>11</v>
       </c>
-      <c r="Y41" s="9"/>
-      <c r="Z41" s="10" t="s">
+      <c r="Y41" s="6"/>
+      <c r="Z41" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="AA41" s="11" t="s">
+      <c r="AA41" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="AB41" s="11"/>
-      <c r="AC41" s="11"/>
-      <c r="AD41" s="10">
+      <c r="AB41" s="8"/>
+      <c r="AC41" s="8"/>
+      <c r="AD41" s="7">
         <v>175</v>
       </c>
-      <c r="AE41" s="10"/>
+      <c r="AE41" s="7"/>
     </row>
     <row r="42" spans="6:31" x14ac:dyDescent="0.25">
       <c r="F42" s="6">
@@ -2918,40 +2921,40 @@
       <c r="M42" s="7">
         <v>3</v>
       </c>
-      <c r="O42" s="9">
+      <c r="O42" s="6">
         <v>12</v>
       </c>
-      <c r="P42" s="9"/>
-      <c r="Q42" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="R42" s="11" t="s">
+      <c r="P42" s="6"/>
+      <c r="Q42" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="R42" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="S42" s="11"/>
-      <c r="T42" s="11"/>
-      <c r="U42" s="10">
+      <c r="S42" s="8"/>
+      <c r="T42" s="8"/>
+      <c r="U42" s="7">
         <v>50</v>
       </c>
-      <c r="V42" s="10">
-        <v>3</v>
-      </c>
-      <c r="X42" s="9">
+      <c r="V42" s="7">
+        <v>3</v>
+      </c>
+      <c r="X42" s="6">
         <v>12</v>
       </c>
-      <c r="Y42" s="9"/>
-      <c r="Z42" s="10" t="s">
+      <c r="Y42" s="6"/>
+      <c r="Z42" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="AA42" s="11" t="s">
+      <c r="AA42" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="AB42" s="11"/>
-      <c r="AC42" s="11"/>
-      <c r="AD42" s="10">
+      <c r="AB42" s="8"/>
+      <c r="AC42" s="8"/>
+      <c r="AD42" s="7">
         <v>175</v>
       </c>
-      <c r="AE42" s="10"/>
+      <c r="AE42" s="7"/>
     </row>
     <row r="43" spans="6:31" x14ac:dyDescent="0.25">
       <c r="F43" s="6">
@@ -2972,22 +2975,22 @@
       <c r="M43" s="7">
         <v>3</v>
       </c>
-      <c r="O43" s="9">
+      <c r="O43" s="6">
         <v>13</v>
       </c>
-      <c r="P43" s="9"/>
-      <c r="Q43" s="10" t="s">
+      <c r="P43" s="6"/>
+      <c r="Q43" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R43" s="11" t="s">
+      <c r="R43" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="S43" s="11"/>
-      <c r="T43" s="11"/>
-      <c r="U43" s="10">
+      <c r="S43" s="8"/>
+      <c r="T43" s="8"/>
+      <c r="U43" s="7">
         <v>75</v>
       </c>
-      <c r="V43" s="10">
+      <c r="V43" s="7">
         <v>3</v>
       </c>
       <c r="X43" s="6">
@@ -3095,12 +3098,17 @@
       <c r="T48" s="1"/>
       <c r="V48" s="2"/>
     </row>
-    <row r="49" spans="17:22" x14ac:dyDescent="0.25">
+    <row r="49" spans="15:22" x14ac:dyDescent="0.25">
       <c r="Q49" s="2"/>
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
       <c r="T49" s="1"/>
       <c r="V49" s="2"/>
+    </row>
+    <row r="55" spans="15:22" x14ac:dyDescent="0.25">
+      <c r="O55" t="s">
+        <v>112</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="138">

</xml_diff>